<commit_message>
feat(docs): affinity estimation com avaliação da equipe 12
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SfTUy7o84Gp6rmVMR2kSC8
</commit_message>
<xml_diff>
--- a/docs/Affinity_Estimation_MultiPag.xlsx
+++ b/docs/Affinity_Estimation_MultiPag.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="117">
   <si>
     <t xml:space="preserve">Affinity Estimation: MultiPag</t>
   </si>
@@ -282,15 +282,15 @@
     <t xml:space="preserve">RF14  Cobranças do cliente por CPF</t>
   </si>
   <si>
+    <t xml:space="preserve">RF25  Validar chave Pix no DICT</t>
+  </si>
+  <si>
     <t xml:space="preserve">RF20  Cliente alterar dados da conta</t>
   </si>
   <si>
     <t xml:space="preserve">RF17  Business excluir a conta</t>
   </si>
   <si>
-    <t xml:space="preserve">RF25  Validar chave Pix no DICT</t>
-  </si>
-  <si>
     <t xml:space="preserve">RF22  Resultado do pagamento</t>
   </si>
   <si>
@@ -315,6 +315,9 @@
     <t xml:space="preserve">Equipe avaliadora:</t>
   </si>
   <si>
+    <t xml:space="preserve">Equipe 12 - WorkForge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Requisito</t>
   </si>
   <si>
@@ -334,6 +337,42 @@
   </si>
   <si>
     <t xml:space="preserve">Decisão da equipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O cadastro parece só um formulário, M não seria suficiente?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O cadastro tem 3 etapas, consulta de CPF e senha com hash. Mantemos L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tem itens, cliente e vários métodos de pagamento, parece maior que XL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O fluxo tem 5 etapas, mas as regras já são conhecidas. Mantemos XL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O extrato tem exportação?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não tem exportação nesta versão, só filtros, paginação e totais. Mantemos L.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A transferência para o banco é real?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A transferência é simulada. Só entram a validação do saldo e da chave e o registro do saque. Mantemos XL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se o DICT demorar ou ficar fora do ar, o que acontece?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acatamos. O tratamento de espera e de nova tentativa dá mais trabalho do que pensamos. Movido para XL.</t>
   </si>
 </sst>
 </file>
@@ -343,7 +382,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -406,6 +445,13 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -531,8 +577,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1473,20 +1519,20 @@
       <c r="D8" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="9"/>
+      <c r="E8" s="8" t="s">
+        <v>86</v>
+      </c>
       <c r="F8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9"/>
       <c r="B9" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="8" t="s">
         <v>88</v>
       </c>
+      <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
     </row>
@@ -1567,7 +1613,9 @@
         <v>96</v>
       </c>
       <c r="B2" s="10"/>
-      <c r="C2" s="11"/>
+      <c r="C2" s="11" t="s">
+        <v>97</v>
+      </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
     </row>
@@ -1576,25 +1624,25 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1608,14 +1656,22 @@
         <f aca="false">'Quadro individual'!F5</f>
         <v>L</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="G5" s="4" t="str">
-        <f aca="false">IF(F5="","",IF(F5="Sim",D5,C5))</f>
-        <v/>
-      </c>
-      <c r="H5" s="5"/>
+        <f aca="false">IF(F5="Sim",D5,C5)</f>
+        <v>L</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
@@ -1632,8 +1688,8 @@
       <c r="E6" s="5"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4" t="str">
-        <f aca="false">IF(F6="","",IF(F6="Sim",D6,C6))</f>
-        <v/>
+        <f aca="false">IF(F6="Sim",D6,C6)</f>
+        <v>M</v>
       </c>
       <c r="H6" s="5"/>
     </row>
@@ -1648,14 +1704,22 @@
         <f aca="false">'Quadro individual'!F7</f>
         <v>XL</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="4"/>
+      <c r="D7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="G7" s="4" t="str">
-        <f aca="false">IF(F7="","",IF(F7="Sim",D7,C7))</f>
-        <v/>
-      </c>
-      <c r="H7" s="5"/>
+        <f aca="false">IF(F7="Sim",D7,C7)</f>
+        <v>XL</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
@@ -1672,8 +1736,8 @@
       <c r="E8" s="5"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="str">
-        <f aca="false">IF(F8="","",IF(F8="Sim",D8,C8))</f>
-        <v/>
+        <f aca="false">IF(F8="Sim",D8,C8)</f>
+        <v>M</v>
       </c>
       <c r="H8" s="5"/>
     </row>
@@ -1692,8 +1756,8 @@
       <c r="E9" s="5"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4" t="str">
-        <f aca="false">IF(F9="","",IF(F9="Sim",D9,C9))</f>
-        <v/>
+        <f aca="false">IF(F9="Sim",D9,C9)</f>
+        <v>S</v>
       </c>
       <c r="H9" s="5"/>
     </row>
@@ -1712,8 +1776,8 @@
       <c r="E10" s="5"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4" t="str">
-        <f aca="false">IF(F10="","",IF(F10="Sim",D10,C10))</f>
-        <v/>
+        <f aca="false">IF(F10="Sim",D10,C10)</f>
+        <v>XS</v>
       </c>
       <c r="H10" s="5"/>
     </row>
@@ -1732,8 +1796,8 @@
       <c r="E11" s="5"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4" t="str">
-        <f aca="false">IF(F11="","",IF(F11="Sim",D11,C11))</f>
-        <v/>
+        <f aca="false">IF(F11="Sim",D11,C11)</f>
+        <v>S</v>
       </c>
       <c r="H11" s="5"/>
     </row>
@@ -1748,16 +1812,24 @@
         <f aca="false">'Quadro individual'!F12</f>
         <v>L</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="4"/>
+      <c r="D12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="G12" s="4" t="str">
-        <f aca="false">IF(F12="","",IF(F12="Sim",D12,C12))</f>
-        <v/>
-      </c>
-      <c r="H12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <f aca="false">IF(F12="Sim",D12,C12)</f>
+        <v>L</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
@@ -1768,14 +1840,22 @@
         <f aca="false">'Quadro individual'!F13</f>
         <v>XL</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="4"/>
+      <c r="D13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="G13" s="4" t="str">
-        <f aca="false">IF(F13="","",IF(F13="Sim",D13,C13))</f>
-        <v/>
-      </c>
-      <c r="H13" s="5"/>
+        <f aca="false">IF(F13="Sim",D13,C13)</f>
+        <v>XL</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
@@ -1792,8 +1872,8 @@
       <c r="E14" s="5"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="str">
-        <f aca="false">IF(F14="","",IF(F14="Sim",D14,C14))</f>
-        <v/>
+        <f aca="false">IF(F14="Sim",D14,C14)</f>
+        <v>M</v>
       </c>
       <c r="H14" s="5"/>
     </row>
@@ -1812,8 +1892,8 @@
       <c r="E15" s="5"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="str">
-        <f aca="false">IF(F15="","",IF(F15="Sim",D15,C15))</f>
-        <v/>
+        <f aca="false">IF(F15="Sim",D15,C15)</f>
+        <v>L</v>
       </c>
       <c r="H15" s="5"/>
     </row>
@@ -1832,8 +1912,8 @@
       <c r="E16" s="5"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4" t="str">
-        <f aca="false">IF(F16="","",IF(F16="Sim",D16,C16))</f>
-        <v/>
+        <f aca="false">IF(F16="Sim",D16,C16)</f>
+        <v>XXL</v>
       </c>
       <c r="H16" s="5"/>
     </row>
@@ -1852,8 +1932,8 @@
       <c r="E17" s="5"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4" t="str">
-        <f aca="false">IF(F17="","",IF(F17="Sim",D17,C17))</f>
-        <v/>
+        <f aca="false">IF(F17="Sim",D17,C17)</f>
+        <v>M</v>
       </c>
       <c r="H17" s="5"/>
     </row>
@@ -1872,8 +1952,8 @@
       <c r="E18" s="5"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="str">
-        <f aca="false">IF(F18="","",IF(F18="Sim",D18,C18))</f>
-        <v/>
+        <f aca="false">IF(F18="Sim",D18,C18)</f>
+        <v>L</v>
       </c>
       <c r="H18" s="5"/>
     </row>
@@ -1892,8 +1972,8 @@
       <c r="E19" s="5"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4" t="str">
-        <f aca="false">IF(F19="","",IF(F19="Sim",D19,C19))</f>
-        <v/>
+        <f aca="false">IF(F19="Sim",D19,C19)</f>
+        <v>XL</v>
       </c>
       <c r="H19" s="5"/>
     </row>
@@ -1912,8 +1992,8 @@
       <c r="E20" s="5"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4" t="str">
-        <f aca="false">IF(F20="","",IF(F20="Sim",D20,C20))</f>
-        <v/>
+        <f aca="false">IF(F20="Sim",D20,C20)</f>
+        <v>S</v>
       </c>
       <c r="H20" s="5"/>
     </row>
@@ -1932,8 +2012,8 @@
       <c r="E21" s="5"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4" t="str">
-        <f aca="false">IF(F21="","",IF(F21="Sim",D21,C21))</f>
-        <v/>
+        <f aca="false">IF(F21="Sim",D21,C21)</f>
+        <v>M</v>
       </c>
       <c r="H21" s="5"/>
     </row>
@@ -1952,8 +2032,8 @@
       <c r="E22" s="5"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="str">
-        <f aca="false">IF(F22="","",IF(F22="Sim",D22,C22))</f>
-        <v/>
+        <f aca="false">IF(F22="Sim",D22,C22)</f>
+        <v>M</v>
       </c>
       <c r="H22" s="5"/>
     </row>
@@ -1972,8 +2052,8 @@
       <c r="E23" s="5"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4" t="str">
-        <f aca="false">IF(F23="","",IF(F23="Sim",D23,C23))</f>
-        <v/>
+        <f aca="false">IF(F23="Sim",D23,C23)</f>
+        <v>S</v>
       </c>
       <c r="H23" s="5"/>
     </row>
@@ -1992,8 +2072,8 @@
       <c r="E24" s="5"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4" t="str">
-        <f aca="false">IF(F24="","",IF(F24="Sim",D24,C24))</f>
-        <v/>
+        <f aca="false">IF(F24="Sim",D24,C24)</f>
+        <v>S</v>
       </c>
       <c r="H24" s="5"/>
     </row>
@@ -2012,8 +2092,8 @@
       <c r="E25" s="5"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4" t="str">
-        <f aca="false">IF(F25="","",IF(F25="Sim",D25,C25))</f>
-        <v/>
+        <f aca="false">IF(F25="Sim",D25,C25)</f>
+        <v>M</v>
       </c>
       <c r="H25" s="5"/>
     </row>
@@ -2032,8 +2112,8 @@
       <c r="E26" s="5"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="str">
-        <f aca="false">IF(F26="","",IF(F26="Sim",D26,C26))</f>
-        <v/>
+        <f aca="false">IF(F26="Sim",D26,C26)</f>
+        <v>S</v>
       </c>
       <c r="H26" s="5"/>
     </row>
@@ -2052,8 +2132,8 @@
       <c r="E27" s="5"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4" t="str">
-        <f aca="false">IF(F27="","",IF(F27="Sim",D27,C27))</f>
-        <v/>
+        <f aca="false">IF(F27="Sim",D27,C27)</f>
+        <v>M</v>
       </c>
       <c r="H27" s="5"/>
     </row>
@@ -2072,12 +2152,12 @@
       <c r="E28" s="5"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4" t="str">
-        <f aca="false">IF(F28="","",IF(F28="Sim",D28,C28))</f>
-        <v/>
+        <f aca="false">IF(F28="Sim",D28,C28)</f>
+        <v>S</v>
       </c>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>62</v>
       </c>
@@ -2088,14 +2168,22 @@
         <f aca="false">'Quadro individual'!F29</f>
         <v>L</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="4"/>
+      <c r="D29" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="G29" s="4" t="str">
-        <f aca="false">IF(F29="","",IF(F29="Sim",D29,C29))</f>
-        <v/>
-      </c>
-      <c r="H29" s="5"/>
+        <f aca="false">IF(F29="Sim",D29,C29)</f>
+        <v>XL</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
@@ -2112,8 +2200,8 @@
       <c r="E30" s="5"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="str">
-        <f aca="false">IF(F30="","",IF(F30="Sim",D30,C30))</f>
-        <v/>
+        <f aca="false">IF(F30="Sim",D30,C30)</f>
+        <v>S</v>
       </c>
       <c r="H30" s="5"/>
     </row>

</xml_diff>